<commit_message>
finish aifinops.dev migration: redirect, remaining refs, docs
Completes the migration so main fully reflects the move.

- functions/_middleware.js: 301-redirect costperacceptedchange.org (and
  www) → aifinops.dev, preserving path + query, before content
  negotiation. Code-complete; no dashboard Redirect Rule required.
- Remaining old-domain references migrated: tools/cpac-cli (README,
  SKILL.md, package.json, src/*.js), scripts/generate-templates.mjs.
- Regenerated public/templates/cpac-tracker.xlsx with the new domain.
- AGENTS.md / README.md / package.json rebranded to AI FinOps (both
  metrics); CHANGELOG entry for the migration + CPAA.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/cpac-tracker.xlsx
+++ b/public/templates/cpac-tracker.xlsx
@@ -30,7 +30,7 @@
         <sz val="10"/>
         <rFont val="Helvetica"/>
       </rPr>
-      <t>Canonical definition at costperacceptedchange.org</t>
+      <t>Canonical definition at aifinops.dev</t>
     </r>
   </si>
   <si>
@@ -88,7 +88,7 @@
     <t>Cost per accepted change — tracker instructions</t>
   </si>
   <si>
-    <t>Canonical definition: https://costperacceptedchange.org</t>
+    <t>Canonical definition: https://aifinops.dev</t>
   </si>
   <si>
     <t>Defined in The Delivery Gap (Brenn Hill, 2026) as the cost vertex of the Verification Triangle.</t>
@@ -166,19 +166,19 @@
     <t>Where to find help</t>
   </si>
   <si>
-    <t>— Definition and worked example: https://costperacceptedchange.org/</t>
-  </si>
-  <si>
-    <t>— How to use the metric correctly: https://costperacceptedchange.org/use</t>
-  </si>
-  <si>
-    <t>— FAQ, including the git command recipe for counting line changes: https://costperacceptedchange.org/faq</t>
-  </si>
-  <si>
-    <t>— Calculator (single-window): https://costperacceptedchange.org/calculator</t>
-  </si>
-  <si>
-    <t>— Quarterly review template: https://costperacceptedchange.org/templates/quarterly-review</t>
+    <t>— Definition and worked example: https://aifinops.dev/</t>
+  </si>
+  <si>
+    <t>— How to use the metric correctly: https://aifinops.dev/use</t>
+  </si>
+  <si>
+    <t>— FAQ, including the git command recipe for counting line changes: https://aifinops.dev/faq</t>
+  </si>
+  <si>
+    <t>— Calculator (single-window): https://aifinops.dev/calculator</t>
+  </si>
+  <si>
+    <t>— Quarterly review template: https://aifinops.dev/templates/quarterly-review</t>
   </si>
   <si>
     <t>— Source: https://github.com/brennhill/cost-per-accepted-change</t>
@@ -1351,7 +1351,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" ht="44" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
         <v>49</v>
       </c>

</xml_diff>

<commit_message>
finish aifinops.dev migration: redirect, remaining refs, docs (#3)
Completes the migration so main fully reflects the move.

- functions/_middleware.js: 301-redirect costperacceptedchange.org (and
  www) → aifinops.dev, preserving path + query, before content
  negotiation. Code-complete; no dashboard Redirect Rule required.
- Remaining old-domain references migrated: tools/cpac-cli (README,
  SKILL.md, package.json, src/*.js), scripts/generate-templates.mjs.
- Regenerated public/templates/cpac-tracker.xlsx with the new domain.
- AGENTS.md / README.md / package.json rebranded to AI FinOps (both
  metrics); CHANGELOG entry for the migration + CPAA.

Co-authored-by: Brenn <brenn@Brenns-MacBook-Pro-2.local>
Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/cpac-tracker.xlsx
+++ b/public/templates/cpac-tracker.xlsx
@@ -30,7 +30,7 @@
         <sz val="10"/>
         <rFont val="Helvetica"/>
       </rPr>
-      <t>Canonical definition at costperacceptedchange.org</t>
+      <t>Canonical definition at aifinops.dev</t>
     </r>
   </si>
   <si>
@@ -88,7 +88,7 @@
     <t>Cost per accepted change — tracker instructions</t>
   </si>
   <si>
-    <t>Canonical definition: https://costperacceptedchange.org</t>
+    <t>Canonical definition: https://aifinops.dev</t>
   </si>
   <si>
     <t>Defined in The Delivery Gap (Brenn Hill, 2026) as the cost vertex of the Verification Triangle.</t>
@@ -166,19 +166,19 @@
     <t>Where to find help</t>
   </si>
   <si>
-    <t>— Definition and worked example: https://costperacceptedchange.org/</t>
-  </si>
-  <si>
-    <t>— How to use the metric correctly: https://costperacceptedchange.org/use</t>
-  </si>
-  <si>
-    <t>— FAQ, including the git command recipe for counting line changes: https://costperacceptedchange.org/faq</t>
-  </si>
-  <si>
-    <t>— Calculator (single-window): https://costperacceptedchange.org/calculator</t>
-  </si>
-  <si>
-    <t>— Quarterly review template: https://costperacceptedchange.org/templates/quarterly-review</t>
+    <t>— Definition and worked example: https://aifinops.dev/</t>
+  </si>
+  <si>
+    <t>— How to use the metric correctly: https://aifinops.dev/use</t>
+  </si>
+  <si>
+    <t>— FAQ, including the git command recipe for counting line changes: https://aifinops.dev/faq</t>
+  </si>
+  <si>
+    <t>— Calculator (single-window): https://aifinops.dev/calculator</t>
+  </si>
+  <si>
+    <t>— Quarterly review template: https://aifinops.dev/templates/quarterly-review</t>
   </si>
   <si>
     <t>— Source: https://github.com/brennhill/cost-per-accepted-change</t>
@@ -1351,7 +1351,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" ht="44" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" ht="22" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
         <v>49</v>
       </c>

</xml_diff>